<commit_message>
docs(tutorials): W-1 updated from the sessions re-run under the revised assistant (diagnosis now finds all three planted faults with a ranked table; corpus examples and engine β in the conceptual answers; report verified); cost table recomputed
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/tutorials/files/w1_build_from_image_after.xlsx
+++ b/docs/tutorials/files/w1_build_from_image_after.xlsx
@@ -3389,13 +3389,15 @@
           <t>Geosynthetic</t>
         </is>
       </c>
-      <c r="H3" s="3" t="str">
-        <f t="shared" ref="H3:H22" si="0">IF($G3="","",IFERROR(VLOOKUP($G3,$AB$8:$AD$11,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="I3" s="3" t="str">
-        <f t="shared" ref="I3:I22" si="1">IF($G3="","",IFERROR(VLOOKUP($G3,$AB$8:$AD$11,3,0),""))</f>
-        <v/>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="J3" s="3">
         <v>800.0</v>
@@ -3462,13 +3464,15 @@
           <t>Geosynthetic</t>
         </is>
       </c>
-      <c r="H4" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I4" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="J4" s="3">
         <v>800.0</v>
@@ -3529,13 +3533,15 @@
           <t>Geosynthetic</t>
         </is>
       </c>
-      <c r="H5" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I5" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="J5" s="3">
         <v>800.0</v>
@@ -3596,13 +3602,15 @@
           <t>Geosynthetic</t>
         </is>
       </c>
-      <c r="H6" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I6" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="J6" s="3">
         <v>800.0</v>
@@ -3660,13 +3668,15 @@
           <t>Geosynthetic</t>
         </is>
       </c>
-      <c r="H7" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I7" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="J7" s="3">
         <v>800.0</v>
@@ -3724,13 +3734,15 @@
           <t>Geosynthetic</t>
         </is>
       </c>
-      <c r="H8" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I8" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="J8" s="3">
         <v>800.0</v>
@@ -10323,7 +10335,7 @@
         <v>10.0</v>
       </c>
       <c r="D10" s="3">
-        <v>-20.0</v>
+        <v>0.0</v>
       </c>
       <c r="E10" s="3">
         <v>0.0</v>
@@ -10413,7 +10425,7 @@
     </row>
     <row r="12" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
-        <v>63.2015621187</v>
+        <v>62.0</v>
       </c>
       <c r="B12" s="3">
         <v>34.0</v>
@@ -10461,13 +10473,13 @@
     </row>
     <row r="13" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
-        <v>33.2015621187</v>
+        <v>32.0</v>
       </c>
       <c r="B13" s="3">
         <v>10.0</v>
       </c>
       <c r="D13" s="3">
-        <v>63.2015621187</v>
+        <v>62.0</v>
       </c>
       <c r="E13" s="3">
         <v>34.0</v>
@@ -10511,7 +10523,7 @@
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="D14" s="3">
-        <v>33.2015621187</v>
+        <v>32.0</v>
       </c>
       <c r="E14" s="3">
         <v>10.0</v>
@@ -10555,7 +10567,7 @@
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="D15" s="3">
-        <v>-20.0</v>
+        <v>0.0</v>
       </c>
       <c r="E15" s="3">
         <v>10.0</v>

</xml_diff>

<commit_message>
tools: assistant suite corpus sweep (--corpus, --resume; scored by input class; 82 of 390 files swept live, 68 pass); sensitivity treats an empty reinforcement list as none; W-1 build-from-drawing re-run under the refusals (1.628, file reopens)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/tutorials/files/w1_build_from_image_after.xlsx
+++ b/docs/tutorials/files/w1_build_from_image_after.xlsx
@@ -3389,15 +3389,13 @@
           <t>Geosynthetic</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="H3" s="3" t="str">
+        <f>IF($G3="","",IFERROR(VLOOKUP($G3,$AB$8:$AD$11,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="I3" s="3" t="str">
+        <f t="shared" ref="I3:I22" si="1">IF($G3="","",IFERROR(VLOOKUP($G3,$AB$8:$AD$11,3,0),""))</f>
+        <v/>
       </c>
       <c r="J3" s="3">
         <v>800.0</v>
@@ -3464,15 +3462,13 @@
           <t>Geosynthetic</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="H4" s="3" t="str">
+        <f>IF($G4="","",IFERROR(VLOOKUP($G4,$AB$8:$AD$11,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="I4" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
       </c>
       <c r="J4" s="3">
         <v>800.0</v>
@@ -3533,15 +3529,13 @@
           <t>Geosynthetic</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="H5" s="3" t="str">
+        <f>IF($G5="","",IFERROR(VLOOKUP($G5,$AB$8:$AD$11,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="I5" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
       </c>
       <c r="J5" s="3">
         <v>800.0</v>
@@ -3602,15 +3596,13 @@
           <t>Geosynthetic</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
-      <c r="I6" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="H6" s="3" t="str">
+        <f>IF($G6="","",IFERROR(VLOOKUP($G6,$AB$8:$AD$11,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="I6" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
       </c>
       <c r="J6" s="3">
         <v>800.0</v>
@@ -3668,15 +3660,13 @@
           <t>Geosynthetic</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
-      <c r="I7" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="H7" s="3" t="str">
+        <f>IF($G7="","",IFERROR(VLOOKUP($G7,$AB$8:$AD$11,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="I7" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
       </c>
       <c r="J7" s="3">
         <v>800.0</v>
@@ -3734,15 +3724,13 @@
           <t>Geosynthetic</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
-      <c r="I8" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="H8" s="3" t="str">
+        <f>IF($G8="","",IFERROR(VLOOKUP($G8,$AB$8:$AD$11,2,0),""))</f>
+        <v/>
+      </c>
+      <c r="I8" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
       </c>
       <c r="J8" s="3">
         <v>800.0</v>
@@ -3794,7 +3782,7 @@
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
       <c r="H9" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF($G9="","",IFERROR(VLOOKUP($G9,$AB$8:$AD$11,2,0),""))</f>
         <v/>
       </c>
       <c r="I9" s="3" t="str">
@@ -3833,7 +3821,7 @@
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
       <c r="H10" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF($G10="","",IFERROR(VLOOKUP($G10,$AB$8:$AD$11,2,0),""))</f>
         <v/>
       </c>
       <c r="I10" s="3" t="str">
@@ -3872,7 +3860,7 @@
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
       <c r="H11" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF($G11="","",IFERROR(VLOOKUP($G11,$AB$8:$AD$11,2,0),""))</f>
         <v/>
       </c>
       <c r="I11" s="3" t="str">
@@ -3911,7 +3899,7 @@
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
       <c r="H12" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF($G12="","",IFERROR(VLOOKUP($G12,$AB$8:$AD$11,2,0),""))</f>
         <v/>
       </c>
       <c r="I12" s="3" t="str">
@@ -3941,7 +3929,7 @@
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
       <c r="H13" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF($G13="","",IFERROR(VLOOKUP($G13,$AB$8:$AD$11,2,0),""))</f>
         <v/>
       </c>
       <c r="I13" s="3" t="str">
@@ -3971,7 +3959,7 @@
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
       <c r="H14" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF($G14="","",IFERROR(VLOOKUP($G14,$AB$8:$AD$11,2,0),""))</f>
         <v/>
       </c>
       <c r="I14" s="3" t="str">
@@ -4001,7 +3989,7 @@
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
       <c r="H15" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF($G15="","",IFERROR(VLOOKUP($G15,$AB$8:$AD$11,2,0),""))</f>
         <v/>
       </c>
       <c r="I15" s="3" t="str">
@@ -4031,7 +4019,7 @@
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
       <c r="H16" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF($G16="","",IFERROR(VLOOKUP($G16,$AB$8:$AD$11,2,0),""))</f>
         <v/>
       </c>
       <c r="I16" s="3" t="str">
@@ -4061,7 +4049,7 @@
       <c r="F17" s="3"/>
       <c r="G17" s="3"/>
       <c r="H17" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF($G17="","",IFERROR(VLOOKUP($G17,$AB$8:$AD$11,2,0),""))</f>
         <v/>
       </c>
       <c r="I17" s="3" t="str">
@@ -4091,7 +4079,7 @@
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
       <c r="H18" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF($G18="","",IFERROR(VLOOKUP($G18,$AB$8:$AD$11,2,0),""))</f>
         <v/>
       </c>
       <c r="I18" s="3" t="str">
@@ -4121,7 +4109,7 @@
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
       <c r="H19" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF($G19="","",IFERROR(VLOOKUP($G19,$AB$8:$AD$11,2,0),""))</f>
         <v/>
       </c>
       <c r="I19" s="3" t="str">
@@ -4151,7 +4139,7 @@
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
       <c r="H20" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF($G20="","",IFERROR(VLOOKUP($G20,$AB$8:$AD$11,2,0),""))</f>
         <v/>
       </c>
       <c r="I20" s="3" t="str">
@@ -4181,7 +4169,7 @@
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
       <c r="H21" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF($G21="","",IFERROR(VLOOKUP($G21,$AB$8:$AD$11,2,0),""))</f>
         <v/>
       </c>
       <c r="I21" s="3" t="str">
@@ -4211,7 +4199,7 @@
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
       <c r="H22" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF($G22="","",IFERROR(VLOOKUP($G22,$AB$8:$AD$11,2,0),""))</f>
         <v/>
       </c>
       <c r="I22" s="3" t="str">
@@ -10425,7 +10413,7 @@
     </row>
     <row r="12" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
-        <v>62.0</v>
+        <v>63.2015621187</v>
       </c>
       <c r="B12" s="3">
         <v>34.0</v>
@@ -10473,13 +10461,13 @@
     </row>
     <row r="13" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
-        <v>32.0</v>
+        <v>33.2015621187</v>
       </c>
       <c r="B13" s="3">
         <v>10.0</v>
       </c>
       <c r="D13" s="3">
-        <v>62.0</v>
+        <v>63.2015621187</v>
       </c>
       <c r="E13" s="3">
         <v>34.0</v>
@@ -10523,7 +10511,7 @@
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="D14" s="3">
-        <v>32.0</v>
+        <v>33.2015621187</v>
       </c>
       <c r="E14" s="3">
         <v>10.0</v>

</xml_diff>

<commit_message>
tutorials(W-1): the LEM-3 sessions re-recorded on Opus 5 under the revised brief and prompts
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/tutorials/files/w1_build_from_image_after.xlsx
+++ b/docs/tutorials/files/w1_build_from_image_after.xlsx
@@ -6698,7 +6698,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Embankment clay</t>
+          <t>Embankment</t>
         </is>
       </c>
       <c r="C11" s="3">
@@ -6796,7 +6796,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Foundation clay</t>
+          <t>Foundation</t>
         </is>
       </c>
       <c r="C12" s="3">
@@ -8717,7 +8717,7 @@
     </row>
     <row r="9" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
-        <v>-30.0</v>
+        <v>0.0</v>
       </c>
       <c r="B9" s="3">
         <v>0.0</v>
@@ -8765,13 +8765,13 @@
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
+        <v>40.0</v>
+      </c>
+      <c r="B10" s="3">
+        <v>20.0</v>
+      </c>
+      <c r="D10" s="3">
         <v>0.0</v>
-      </c>
-      <c r="B10" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="D10" s="3">
-        <v>90.0</v>
       </c>
       <c r="E10" s="3">
         <v>0.0</v>
@@ -8813,13 +8813,17 @@
     </row>
     <row r="11" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
-        <v>40.0</v>
+        <v>90.0</v>
       </c>
       <c r="B11" s="3">
         <v>20.0</v>
       </c>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
+      <c r="D11" s="3">
+        <v>90.0</v>
+      </c>
+      <c r="E11" s="3">
+        <v>0.0</v>
+      </c>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
       <c r="J11" s="3"/>
@@ -8856,12 +8860,8 @@
       <c r="AR11" s="19"/>
     </row>
     <row r="12" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A12" s="3">
-        <v>90.0</v>
-      </c>
-      <c r="B12" s="3">
-        <v>20.0</v>
-      </c>
+      <c r="A12" s="3"/>
+      <c r="B12" s="3"/>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
       <c r="G12" s="3"/>

</xml_diff>

<commit_message>
tutorials(W-1): the build session shows the whole Studio window — model on the canvas, conversation in the dock; recorder gains a window grab
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/tutorials/files/w1_build_from_image_after.xlsx
+++ b/docs/tutorials/files/w1_build_from_image_after.xlsx
@@ -6704,7 +6704,9 @@
       <c r="C11" s="3">
         <v>130.0</v>
       </c>
-      <c r="D11" s="3"/>
+      <c r="D11" s="3">
+        <v>130.0</v>
+      </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
           <t>mc</t>
@@ -6802,7 +6804,9 @@
       <c r="C12" s="3">
         <v>135.0</v>
       </c>
-      <c r="D12" s="3"/>
+      <c r="D12" s="3">
+        <v>135.0</v>
+      </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
           <t>mc</t>
@@ -8717,7 +8721,7 @@
     </row>
     <row r="9" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
-        <v>0.0</v>
+        <v>-30.0</v>
       </c>
       <c r="B9" s="3">
         <v>0.0</v>
@@ -8765,13 +8769,13 @@
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
-        <v>40.0</v>
+        <v>0.0</v>
       </c>
       <c r="B10" s="3">
-        <v>20.0</v>
+        <v>0.0</v>
       </c>
       <c r="D10" s="3">
-        <v>0.0</v>
+        <v>90.0</v>
       </c>
       <c r="E10" s="3">
         <v>0.0</v>
@@ -8813,17 +8817,13 @@
     </row>
     <row r="11" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
-        <v>90.0</v>
+        <v>40.0</v>
       </c>
       <c r="B11" s="3">
         <v>20.0</v>
       </c>
-      <c r="D11" s="3">
-        <v>90.0</v>
-      </c>
-      <c r="E11" s="3">
-        <v>0.0</v>
-      </c>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
       <c r="J11" s="3"/>
@@ -8860,8 +8860,12 @@
       <c r="AR11" s="19"/>
     </row>
     <row r="12" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
+      <c r="A12" s="3">
+        <v>90.0</v>
+      </c>
+      <c r="B12" s="3">
+        <v>20.0</v>
+      </c>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
       <c r="G12" s="3"/>

</xml_diff>